<commit_message>
Weapon 및 RandomBox 관련 데이터파싱
WeaponData 구조 변경
Localization을 별도의 Json 파일이 아닌
Weapons.json에서 읽도록 변경
Rarities를 별도 json으로 추출
gacha_tables.json 추가
</commit_message>
<xml_diff>
--- a/Content/Data/WeaponData.xlsx
+++ b/Content/Data/WeaponData.xlsx
@@ -8,14 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeaponTypes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rarity" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Localization" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pistol" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssaultRifle" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SniperRifle" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SubMachineGun" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShotGun" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Localization" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pistol" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssaultRifle" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SniperRifle" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SubMachineGun" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShotGun" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -236,12 +235,90 @@
     <author>Weapon Data Schema</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>이 시트의 TypeID는 각 무기 타입 시트 이름과 반드시 일치해야 합니다.
-(예: 'Pistol' 시트가 있으면 여기에도 TypeID='Pistol' 행이 있어야 함)
-새로운 무기 카테고리(Sword, Bow, Spear 등)를 추가할 때도
-이 시트에 행을 먼저 추가한 뒤, 같은 이름의 시트를 만들면 됩니다.</t>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>등급 값 (Common/Rare/Epic). 실제 정의(DropWeight/SellValue 등)는 RandomBox.xlsx의 Rarity 시트가 유일한 출처.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>발당(펠릿당) 데미지. 총 데미지 = Damage x PelletCount.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>한 번 발사에 판정되는 펠릿 수. 일반 무기는 1, ShotGun만 1보다 큼.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>초당 발사 횟수(RPS). FireInterval = 1 / FireRate_RPS
+FireMode=Burst인 경우: 버스트와 버스트 사이 재사격 간격을 의미.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>발사 방식: Single / Burst / FullAuto</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>FireMode=Burst일 때만 의미 있는 값. 그 외에는 0.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Burst 내부 발사 간격(초). FireRate_RPS(버스트간 간격)와 별개. 그 외에는 0.</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>TRUE=히트스캔, FALSE=투사체.</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능.</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>조준경/가늠자 배율. 조준경 없으면 1.0.</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>무조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0" shapeId="0">
+      <text>
+        <t>예약 필드 (현재 미사용). 추후 카메라 반동 전환 시 사용 예정.</t>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <t>예약 필드 (현재 미사용). RecoilVertical과 동일 목적.</t>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="0" shapeId="0">
+      <text>
+        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier와 별개로 조준 시 추가 적용.</t>
       </text>
     </comment>
   </commentList>
@@ -254,12 +331,90 @@
     <author>Weapon Data Schema</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>이 시트의 RarityID는 Weapon 시트의 Rarity 컬럼 값과 반드시 일치해야 합니다.
-DropWeight: 랜덤 무기상자/맵 스폰에서 이 등급이 뽑힐 상대 가중치.
-SellValue: 이 등급 무기를 판매할 때 지급되는 고정 크레딧 값
-(무기 개별 판매가는 없고, 등급의 SellValue를 그대로 사용).</t>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>등급 값 (Common/Rare/Epic). 실제 정의(DropWeight/SellValue 등)는 RandomBox.xlsx의 Rarity 시트가 유일한 출처.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>발당(펠릿당) 데미지. 총 데미지 = Damage x PelletCount.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>한 번 발사에 판정되는 펠릿 수. 일반 무기는 1, ShotGun만 1보다 큼.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>초당 발사 횟수(RPS). FireInterval = 1 / FireRate_RPS
+FireMode=Burst인 경우: 버스트와 버스트 사이 재사격 간격을 의미.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>발사 방식: Single / Burst / FullAuto</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>FireMode=Burst일 때만 의미 있는 값. 그 외에는 0.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Burst 내부 발사 간격(초). FireRate_RPS(버스트간 간격)와 별개. 그 외에는 0.</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>TRUE=히트스캔, FALSE=투사체.</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능.</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>조준경/가늠자 배율. 조준경 없으면 1.0.</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>무조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0" shapeId="0">
+      <text>
+        <t>예약 필드 (현재 미사용). 추후 카메라 반동 전환 시 사용 예정.</t>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <t>예약 필드 (현재 미사용). RecoilVertical과 동일 목적.</t>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="0" shapeId="0">
+      <text>
+        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier와 별개로 조준 시 추가 적용.</t>
       </text>
     </comment>
   </commentList>
@@ -272,11 +427,90 @@
     <author>Weapon Data Schema</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Weapon 시트의 NameKey/DescKey가 참조하는 키.
-언어를 추가하려면 오른쪽에 컬럼(예: ja, zh-Hans)만 추가하면 됨.
-모든 언어 컬럼에 빈 칸이 없어야 컨버터 검증을 통과함.</t>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>등급 값 (Common/Rare/Epic). 실제 정의(DropWeight/SellValue 등)는 RandomBox.xlsx의 Rarity 시트가 유일한 출처.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>발당(펠릿당) 데미지. 총 데미지 = Damage x PelletCount.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>한 번 발사에 판정되는 펠릿 수. 일반 무기는 1, ShotGun만 1보다 큼.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>초당 발사 횟수(RPS). FireInterval = 1 / FireRate_RPS
+FireMode=Burst인 경우: 버스트와 버스트 사이 재사격 간격을 의미.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>발사 방식: Single / Burst / FullAuto</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>FireMode=Burst일 때만 의미 있는 값. 그 외에는 0.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Burst 내부 발사 간격(초). FireRate_RPS(버스트간 간격)와 별개. 그 외에는 0.</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>TRUE=히트스캔, FALSE=투사체.</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능.</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>조준경/가늠자 배율. 조준경 없으면 1.0.</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>무조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0" shapeId="0">
+      <text>
+        <t>예약 필드 (현재 미사용). 추후 카메라 반동 전환 시 사용 예정.</t>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <t>예약 필드 (현재 미사용). RecoilVertical과 동일 목적.</t>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="0" shapeId="0">
+      <text>
+        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier와 별개로 조준 시 추가 적용.</t>
       </text>
     </comment>
   </commentList>
@@ -289,99 +523,90 @@
     <author>Weapon Data Schema</author>
   </authors>
   <commentList>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>등급 값 (Common/Rare/Epic). 실제 정의(DropWeight/SellValue 등)는 RandomBox.xlsx의 Rarity 시트가 유일한 출처.</t>
+      </text>
+    </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Name (예: P_1.Name)
-Localization 시트에 이 키와 각 언어 컬럼 값이 있어야 함.</t>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Description (예: P_1.Description)</t>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>발당(펠릿당) 데미지. 실제 총 데미지 = Damage x PelletCount.
-일반 무기는 PelletCount=1이라 사실상 Damage가 곧 총 데미지.</t>
+        <t>발당(펠릿당) 데미지. 총 데미지 = Damage x PelletCount.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>한 번 발사에 판정되는 펠릿(투사체) 수.
-일반 무기는 1로 고정, ShotGun처럼 산탄이 여러 개인 무기만 1보다 큼.</t>
+        <t>한 번 발사에 판정되는 펠릿 수. 일반 무기는 1, ShotGun만 1보다 큼.</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>초당 발사 횟수(RPS) 기준.
-언리얼 발사 간격 계산: FireInterval = 1 / FireRate_RPS
-예: SR_1 = 0.67 (약 1.5초에 1발, 볼트액션)
-FireMode=Burst인 경우: '버스트와 버스트 사이' 재사격 간격을 의미함
-(버스트 내부 발사 간격은 BurstShotInterval 사용).</t>
+        <t>초당 발사 횟수(RPS). FireInterval = 1 / FireRate_RPS
+FireMode=Burst인 경우: 버스트와 버스트 사이 재사격 간격을 의미.</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>발사 방식. 값: Single / Burst / FullAuto</t>
+        <t>발사 방식: Single / Burst / FullAuto</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>FireMode=Burst일 때만 의미 있는 값. 그 외 FireMode에서는 0.</t>
+        <t>FireMode=Burst일 때만 의미 있는 값. 그 외에는 0.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>FireMode=Burst일 때, 버스트 '내부'에서 한 발과 다음 발 사이의 간격(초).
-FireRate_RPS(버스트간 간격)와는 별개 값. 그 외 FireMode에서는 0.</t>
+        <t>Burst 내부 발사 간격(초). FireRate_RPS(버스트간 간격)와 별개. 그 외에는 0.</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>TRUE = 히트스캔 판정, FALSE = 투사체(Projectile) 판정.
-FALSE인 경우 ProjectileSpeed 값이 반드시 필요.</t>
+        <t>TRUE=히트스캔, FALSE=투사체.</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
-        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능 (예: 추후 추가될 일부 근접무기).</t>
+        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능.</t>
       </text>
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
-        <t>조준경/가늠자 배율. 조준경이 없는 무기는 1.0(배율 없음)으로 설정.
-예: SR_1 = 6.0 (6배율 스코프), 일반 소총 = 1.0~2.0 (기계식/도트/저배율).</t>
+        <t>조준경/가늠자 배율. 조준경 없으면 1.0.</t>
       </text>
     </comment>
     <comment ref="Z1" authorId="0" shapeId="0">
       <text>
-        <t>무조준(Hipfire) 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
+        <t>무조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
       </text>
     </comment>
     <comment ref="AA1" authorId="0" shapeId="0">
       <text>
-        <t>조준(ADS) 상태에서 탄퍼짐이 도달할 수 있는 최대치 (보통 Hipfire보다 작음).</t>
+        <t>조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
       </text>
     </comment>
     <comment ref="AD1" authorId="0" shapeId="0">
       <text>
-        <t>예약 필드 (현재 미사용)
-현재는 탄퍼짐(bloom) 기반 반동만 사용 중.
-추후 카메라/에임 이동형 반동으로 밸런싱 전환 시 사용 예정.
-지금은 0으로 두거나 공란으로 둘 것.</t>
+        <t>예약 필드 (현재 미사용). 추후 카메라 반동 전환 시 사용 예정.</t>
       </text>
     </comment>
     <comment ref="AE1" authorId="0" shapeId="0">
       <text>
-        <t>예약 필드 (현재 미사용) - RecoilVertical과 동일한 목적.</t>
+        <t>예약 필드 (현재 미사용). RecoilVertical과 동일 목적.</t>
       </text>
     </comment>
     <comment ref="AG1" authorId="0" shapeId="0">
       <text>
-        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier(장착 중 기본 이동속도)와는 별개로, 조준 시 추가로 적용됨.</t>
+        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier와 별개로 조준 시 추가 적용.</t>
       </text>
     </comment>
   </commentList>
@@ -394,414 +619,90 @@
     <author>Weapon Data Schema</author>
   </authors>
   <commentList>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>등급 값 (Common/Rare/Epic). 실제 정의(DropWeight/SellValue 등)는 RandomBox.xlsx의 Rarity 시트가 유일한 출처.</t>
+      </text>
+    </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Name (예: P_1.Name)
-Localization 시트에 이 키와 각 언어 컬럼 값이 있어야 함.</t>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Description (예: P_1.Description)</t>
+        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>발당(펠릿당) 데미지. 실제 총 데미지 = Damage x PelletCount.
-일반 무기는 PelletCount=1이라 사실상 Damage가 곧 총 데미지.</t>
+        <t>발당(펠릿당) 데미지. 총 데미지 = Damage x PelletCount.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>한 번 발사에 판정되는 펠릿(투사체) 수.
-일반 무기는 1로 고정, ShotGun처럼 산탄이 여러 개인 무기만 1보다 큼.</t>
+        <t>한 번 발사에 판정되는 펠릿 수. 일반 무기는 1, ShotGun만 1보다 큼.</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>초당 발사 횟수(RPS) 기준.
-언리얼 발사 간격 계산: FireInterval = 1 / FireRate_RPS
-예: SR_1 = 0.67 (약 1.5초에 1발, 볼트액션)
-FireMode=Burst인 경우: '버스트와 버스트 사이' 재사격 간격을 의미함
-(버스트 내부 발사 간격은 BurstShotInterval 사용).</t>
+        <t>초당 발사 횟수(RPS). FireInterval = 1 / FireRate_RPS
+FireMode=Burst인 경우: 버스트와 버스트 사이 재사격 간격을 의미.</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>발사 방식. 값: Single / Burst / FullAuto</t>
+        <t>발사 방식: Single / Burst / FullAuto</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>FireMode=Burst일 때만 의미 있는 값. 그 외 FireMode에서는 0.</t>
+        <t>FireMode=Burst일 때만 의미 있는 값. 그 외에는 0.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>FireMode=Burst일 때, 버스트 '내부'에서 한 발과 다음 발 사이의 간격(초).
-FireRate_RPS(버스트간 간격)와는 별개 값. 그 외 FireMode에서는 0.</t>
+        <t>Burst 내부 발사 간격(초). FireRate_RPS(버스트간 간격)와 별개. 그 외에는 0.</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>TRUE = 히트스캔 판정, FALSE = 투사체(Projectile) 판정.
-FALSE인 경우 ProjectileSpeed 값이 반드시 필요.</t>
+        <t>TRUE=히트스캔, FALSE=투사체.</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
-        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능 (예: 추후 추가될 일부 근접무기).</t>
+        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능.</t>
       </text>
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
-        <t>조준경/가늠자 배율. 조준경이 없는 무기는 1.0(배율 없음)으로 설정.
-예: SR_1 = 6.0 (6배율 스코프), 일반 소총 = 1.0~2.0 (기계식/도트/저배율).</t>
+        <t>조준경/가늠자 배율. 조준경 없으면 1.0.</t>
       </text>
     </comment>
     <comment ref="Z1" authorId="0" shapeId="0">
       <text>
-        <t>무조준(Hipfire) 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
+        <t>무조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
       </text>
     </comment>
     <comment ref="AA1" authorId="0" shapeId="0">
       <text>
-        <t>조준(ADS) 상태에서 탄퍼짐이 도달할 수 있는 최대치 (보통 Hipfire보다 작음).</t>
+        <t>조준 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
       </text>
     </comment>
     <comment ref="AD1" authorId="0" shapeId="0">
       <text>
-        <t>예약 필드 (현재 미사용)
-현재는 탄퍼짐(bloom) 기반 반동만 사용 중.
-추후 카메라/에임 이동형 반동으로 밸런싱 전환 시 사용 예정.
-지금은 0으로 두거나 공란으로 둘 것.</t>
+        <t>예약 필드 (현재 미사용). 추후 카메라 반동 전환 시 사용 예정.</t>
       </text>
     </comment>
     <comment ref="AE1" authorId="0" shapeId="0">
       <text>
-        <t>예약 필드 (현재 미사용) - RecoilVertical과 동일한 목적.</t>
+        <t>예약 필드 (현재 미사용). RecoilVertical과 동일 목적.</t>
       </text>
     </comment>
     <comment ref="AG1" authorId="0" shapeId="0">
       <text>
-        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier(장착 중 기본 이동속도)와는 별개로, 조준 시 추가로 적용됨.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Weapon Data Schema</author>
-  </authors>
-  <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Name (예: P_1.Name)
-Localization 시트에 이 키와 각 언어 컬럼 값이 있어야 함.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Description (예: P_1.Description)</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>발당(펠릿당) 데미지. 실제 총 데미지 = Damage x PelletCount.
-일반 무기는 PelletCount=1이라 사실상 Damage가 곧 총 데미지.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>한 번 발사에 판정되는 펠릿(투사체) 수.
-일반 무기는 1로 고정, ShotGun처럼 산탄이 여러 개인 무기만 1보다 큼.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>초당 발사 횟수(RPS) 기준.
-언리얼 발사 간격 계산: FireInterval = 1 / FireRate_RPS
-예: SR_1 = 0.67 (약 1.5초에 1발, 볼트액션)
-FireMode=Burst인 경우: '버스트와 버스트 사이' 재사격 간격을 의미함
-(버스트 내부 발사 간격은 BurstShotInterval 사용).</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>발사 방식. 값: Single / Burst / FullAuto</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>FireMode=Burst일 때만 의미 있는 값. 그 외 FireMode에서는 0.</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>FireMode=Burst일 때, 버스트 '내부'에서 한 발과 다음 발 사이의 간격(초).
-FireRate_RPS(버스트간 간격)와는 별개 값. 그 외 FireMode에서는 0.</t>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <t>TRUE = 히트스캔 판정, FALSE = 투사체(Projectile) 판정.
-FALSE인 경우 ProjectileSpeed 값이 반드시 필요.</t>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능 (예: 추후 추가될 일부 근접무기).</t>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <t>조준경/가늠자 배율. 조준경이 없는 무기는 1.0(배율 없음)으로 설정.
-예: SR_1 = 6.0 (6배율 스코프), 일반 소총 = 1.0~2.0 (기계식/도트/저배율).</t>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <t>무조준(Hipfire) 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
-      </text>
-    </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 상태에서 탄퍼짐이 도달할 수 있는 최대치 (보통 Hipfire보다 작음).</t>
-      </text>
-    </comment>
-    <comment ref="AD1" authorId="0" shapeId="0">
-      <text>
-        <t>예약 필드 (현재 미사용)
-현재는 탄퍼짐(bloom) 기반 반동만 사용 중.
-추후 카메라/에임 이동형 반동으로 밸런싱 전환 시 사용 예정.
-지금은 0으로 두거나 공란으로 둘 것.</t>
-      </text>
-    </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
-      <text>
-        <t>예약 필드 (현재 미사용) - RecoilVertical과 동일한 목적.</t>
-      </text>
-    </comment>
-    <comment ref="AG1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier(장착 중 기본 이동속도)와는 별개로, 조준 시 추가로 적용됨.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Weapon Data Schema</author>
-  </authors>
-  <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Name (예: P_1.Name)
-Localization 시트에 이 키와 각 언어 컬럼 값이 있어야 함.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Description (예: P_1.Description)</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>발당(펠릿당) 데미지. 실제 총 데미지 = Damage x PelletCount.
-일반 무기는 PelletCount=1이라 사실상 Damage가 곧 총 데미지.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>한 번 발사에 판정되는 펠릿(투사체) 수.
-일반 무기는 1로 고정, ShotGun처럼 산탄이 여러 개인 무기만 1보다 큼.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>초당 발사 횟수(RPS) 기준.
-언리얼 발사 간격 계산: FireInterval = 1 / FireRate_RPS
-예: SR_1 = 0.67 (약 1.5초에 1발, 볼트액션)
-FireMode=Burst인 경우: '버스트와 버스트 사이' 재사격 간격을 의미함
-(버스트 내부 발사 간격은 BurstShotInterval 사용).</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>발사 방식. 값: Single / Burst / FullAuto</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>FireMode=Burst일 때만 의미 있는 값. 그 외 FireMode에서는 0.</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>FireMode=Burst일 때, 버스트 '내부'에서 한 발과 다음 발 사이의 간격(초).
-FireRate_RPS(버스트간 간격)와는 별개 값. 그 외 FireMode에서는 0.</t>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <t>TRUE = 히트스캔 판정, FALSE = 투사체(Projectile) 판정.
-FALSE인 경우 ProjectileSpeed 값이 반드시 필요.</t>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능 (예: 추후 추가될 일부 근접무기).</t>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <t>조준경/가늠자 배율. 조준경이 없는 무기는 1.0(배율 없음)으로 설정.
-예: SR_1 = 6.0 (6배율 스코프), 일반 소총 = 1.0~2.0 (기계식/도트/저배율).</t>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <t>무조준(Hipfire) 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
-      </text>
-    </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 상태에서 탄퍼짐이 도달할 수 있는 최대치 (보통 Hipfire보다 작음).</t>
-      </text>
-    </comment>
-    <comment ref="AD1" authorId="0" shapeId="0">
-      <text>
-        <t>예약 필드 (현재 미사용)
-현재는 탄퍼짐(bloom) 기반 반동만 사용 중.
-추후 카메라/에임 이동형 반동으로 밸런싱 전환 시 사용 예정.
-지금은 0으로 두거나 공란으로 둘 것.</t>
-      </text>
-    </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
-      <text>
-        <t>예약 필드 (현재 미사용) - RecoilVertical과 동일한 목적.</t>
-      </text>
-    </comment>
-    <comment ref="AG1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier(장착 중 기본 이동속도)와는 별개로, 조준 시 추가로 적용됨.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Weapon Data Schema</author>
-  </authors>
-  <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Name (예: P_1.Name)
-Localization 시트에 이 키와 각 언어 컬럼 값이 있어야 함.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>실제 텍스트가 아니라 Localization 시트를 참조하는 키.
-형식: {Index}.Description (예: P_1.Description)</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>발당(펠릿당) 데미지. 실제 총 데미지 = Damage x PelletCount.
-일반 무기는 PelletCount=1이라 사실상 Damage가 곧 총 데미지.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>한 번 발사에 판정되는 펠릿(투사체) 수.
-일반 무기는 1로 고정, ShotGun처럼 산탄이 여러 개인 무기만 1보다 큼.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>초당 발사 횟수(RPS) 기준.
-언리얼 발사 간격 계산: FireInterval = 1 / FireRate_RPS
-예: SR_1 = 0.67 (약 1.5초에 1발, 볼트액션)
-FireMode=Burst인 경우: '버스트와 버스트 사이' 재사격 간격을 의미함
-(버스트 내부 발사 간격은 BurstShotInterval 사용).</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>발사 방식. 값: Single / Burst / FullAuto</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>FireMode=Burst일 때만 의미 있는 값. 그 외 FireMode에서는 0.</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>FireMode=Burst일 때, 버스트 '내부'에서 한 발과 다음 발 사이의 간격(초).
-FireRate_RPS(버스트간 간격)와는 별개 값. 그 외 FireMode에서는 0.</t>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <t>TRUE = 히트스캔 판정, FALSE = 투사체(Projectile) 판정.
-FALSE인 경우 ProjectileSpeed 값이 반드시 필요.</t>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능 (예: 추후 추가될 일부 근접무기).</t>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <t>조준경/가늠자 배율. 조준경이 없는 무기는 1.0(배율 없음)으로 설정.
-예: SR_1 = 6.0 (6배율 스코프), 일반 소총 = 1.0~2.0 (기계식/도트/저배율).</t>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <t>무조준(Hipfire) 상태에서 탄퍼짐이 도달할 수 있는 최대치.</t>
-      </text>
-    </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 상태에서 탄퍼짐이 도달할 수 있는 최대치 (보통 Hipfire보다 작음).</t>
-      </text>
-    </comment>
-    <comment ref="AD1" authorId="0" shapeId="0">
-      <text>
-        <t>예약 필드 (현재 미사용)
-현재는 탄퍼짐(bloom) 기반 반동만 사용 중.
-추후 카메라/에임 이동형 반동으로 밸런싱 전환 시 사용 예정.
-지금은 0으로 두거나 공란으로 둘 것.</t>
-      </text>
-    </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
-      <text>
-        <t>예약 필드 (현재 미사용) - RecoilVertical과 동일한 목적.</t>
-      </text>
-    </comment>
-    <comment ref="AG1" authorId="0" shapeId="0">
-      <text>
-        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier(장착 중 기본 이동속도)와는 별개로, 조준 시 추가로 적용됨.</t>
+        <t>조준(ADS) 중 이동속도 배율. MoveSpeedMultiplier와 별개로 조준 시 추가 적용.</t>
       </text>
     </comment>
   </commentList>
@@ -1108,7 +1009,7 @@
     <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TypeID</t>
@@ -1135,7 +1036,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="14" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>string</t>
@@ -1299,157 +1200,10 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00FFC000"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13.2" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>RarityID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>DisplayName</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>DropWeight</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SellValue</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>#B0B0B0</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>희귀</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>#3B82F6</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>영웅</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>#A855F7</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>800</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0000B0F0"/>
@@ -1464,7 +1218,7 @@
     <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Key</t>
@@ -1608,12 +1362,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>장거리에서 원샷킬을 노릴 수 있는 볼트액션 저격소총.</t>
+          <t>장거리에서 원샷킬을 노릴 수 있는 저격소총.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>A bolt-action sniper rifle capable of long-range one-shot kills.</t>
+          <t>A sniper rifle capable of long-range one-shot kills.</t>
         </is>
       </c>
     </row>
@@ -1687,11 +1441,10 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="008EA9DB"/>
@@ -2216,11 +1969,8 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="S3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="U3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="S3 U3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -2238,7 +1988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0070AD47"/>
@@ -2886,11 +2636,8 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="S3:S4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="U3:U4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="S3:S4 U3:U4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="B3:B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -2908,7 +2655,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>
@@ -3433,11 +3180,8 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="S3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="U3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="S3 U3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -3455,7 +3199,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00BF8F00"/>
@@ -3980,11 +3724,8 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="S3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="U3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="S3 U3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -4002,7 +3743,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -4541,11 +4282,8 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="S3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="U3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="S3 U3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -4563,7 +4301,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4575,7 +4313,7 @@
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4618,7 +4356,7 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>고유 인덱스. 예: P_1, AR_1, AR_2, SR_1, SMG_1, SG_1. 절대 변경 금지.</t>
+          <t>고유 인덱스. 절대 변경 금지.</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4378,7 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>해당 시트에 고정된 타입 값 (Pistol/AssaultRifle/SniperRifle/SubMachineGun/ShotGun).</t>
+          <t>해당 시트에 고정된 타입 값.</t>
         </is>
       </c>
     </row>
@@ -4662,7 +4400,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Rarity 마스터 시트 참조 (Common/Rare/Epic). 판매가는 Rarity.SellValue 사용, Weapon엔 별도 CreditValue 없음.</t>
+          <t>등급 값 (Common/Rare/Epic). 실제 정의는 RandomBox.xlsx의 Rarity 시트.</t>
         </is>
       </c>
     </row>
@@ -4684,7 +4422,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>인게임 표시 이름의 로컬라이징 키. 실제 문자열은 Localization 시트에서 관리.</t>
+          <t>로컬라이징 키 (표시 이름).</t>
         </is>
       </c>
     </row>
@@ -4706,7 +4444,7 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>UI 설명 텍스트의 로컬라이징 키. 실제 문자열은 Localization 시트에서 관리.</t>
+          <t>로컬라이징 키 (설명).</t>
         </is>
       </c>
     </row>
@@ -4750,7 +4488,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>한 번 발사에 판정되는 펠릿 수. 일반 무기는 1, ShotGun만 1보다 큼.</t>
+          <t>한 번 발사에 판정되는 펠릿 수.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4532,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>초당 발사 횟수(RPS). FireInterval = 1 / FireRate_RPS. Burst에서는 버스트간 간격.</t>
+          <t>초당 발사 횟수(RPS). Burst에서는 버스트간 간격.</t>
         </is>
       </c>
     </row>
@@ -4838,7 +4576,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>FireMode=Burst일 때만 의미 있는 값. 그 외 FireMode에서는 0.</t>
+          <t>FireMode=Burst일 때만 의미 있는 값.</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4598,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Burst 내부 발사 간격(초). FireRate_RPS(버스트간 간격)와 별개. 그 외에는 0.</t>
+          <t>Burst 내부 발사 간격(초).</t>
         </is>
       </c>
     </row>
@@ -4948,7 +4686,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>데미지 감소가 시작되는 거리.</t>
+          <t>데미지 감소 시작 거리.</t>
         </is>
       </c>
     </row>
@@ -4992,7 +4730,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>MaxRange 도달 시 최소 데미지.</t>
+          <t>최소 데미지.</t>
         </is>
       </c>
     </row>
@@ -5036,7 +4774,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>투사체 속도. Hitscan이면 0.</t>
+          <t>투사체 속도.</t>
         </is>
       </c>
     </row>
@@ -5058,7 +4796,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>조준(ADS) 가능 여부. FALSE면 이 무기는 조준 자체가 불가능.</t>
+          <t>조준(ADS) 가능 여부.</t>
         </is>
       </c>
     </row>
@@ -5080,7 +4818,7 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>조준경/가늠자 배율. 조준경 없으면 1.0.</t>
+          <t>조준경 배율. 없으면 1.0.</t>
         </is>
       </c>
     </row>
@@ -5102,7 +4840,7 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>무조준 상태 탄착 분산도(기본값).</t>
+          <t>무조준 탄착 분산도.</t>
         </is>
       </c>
     </row>
@@ -5124,7 +4862,7 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>조준(ADS) 상태 탄착 분산도(기본값).</t>
+          <t>조준 탄착 분산도.</t>
         </is>
       </c>
     </row>
@@ -5168,7 +4906,7 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>무조준 상태에서 탄퍼짐 최대 한계치.</t>
+          <t>무조준 탄퍼짐 최대치.</t>
         </is>
       </c>
     </row>
@@ -5190,7 +4928,7 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>조준 상태에서 탄퍼짐 최대 한계치 (보통 Hipfire보다 작음).</t>
+          <t>조준 탄퍼짐 최대치.</t>
         </is>
       </c>
     </row>
@@ -5212,7 +4950,7 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>사격 정지 후 탄퍼짐 회복 시작까지 딜레이(초).</t>
+          <t>탄퍼짐 회복 시작 딜레이(초).</t>
         </is>
       </c>
     </row>
@@ -5256,7 +4994,7 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>현재 미사용. 추후 카메라 반동 도입 시 사용 예정 필드.</t>
+          <t>미사용.</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5016,7 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>현재 미사용. 추후 카메라 반동 도입 시 사용 예정 필드.</t>
+          <t>미사용.</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5038,7 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>조준(ADS) 전환 소요 시간(초).</t>
+          <t>조준 전환 소요 시간(초).</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5060,7 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>조준(ADS) 중 이동속도 배율.</t>
+          <t>조준 중 이동속도 배율.</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5082,7 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>무기 장착 중 기본 이동속도 배율.</t>
+          <t>장착 중 기본 이동속도 배율.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5104,7 @@
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>무기 교체(꺼내기) 소요 시간(초).</t>
+          <t>무기 교체 소요 시간(초).</t>
         </is>
       </c>
     </row>

</xml_diff>